<commit_message>
fixes suspension arm cad
</commit_message>
<xml_diff>
--- a/Suspension/3D_Suspension_Analyzer/3D_Suspension_Analyzer_V2.xlsx
+++ b/Suspension/3D_Suspension_Analyzer/3D_Suspension_Analyzer_V2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\share\OneDrive\Documents\Personal Projects\GOGO Kart\CAD\GOGO_KART_FSAE\Suspension\3D_Suspension_Analyzer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{11981329-2FBF-411D-AAC5-D9B3FE8083FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{E348518A-BE35-44ED-B240-FC9E1B5B3338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Suspension Analyzer" sheetId="1" r:id="rId1"/>
@@ -11699,7 +11699,7 @@
         <v>221</v>
       </c>
       <c r="J17" s="24">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="K17" s="24" t="s">
         <v>222</v>
@@ -11803,7 +11803,7 @@
       </c>
       <c r="J22" s="25">
         <f>(J13*9.8)*(J14+J17*J16)/(J14+J15)</f>
-        <v>2440.9602852492494</v>
+        <v>2383.4644327059054</v>
       </c>
       <c r="K22" s="24" t="s">
         <v>227</v>
@@ -11825,7 +11825,7 @@
       </c>
       <c r="J23" s="25">
         <f>(J13*9.8)*(J15-J17*J16)/(J14+J15)</f>
-        <v>730.02309744427953</v>
+        <v>787.51894998762373</v>
       </c>
       <c r="K23" s="24" t="s">
         <v>227</v>
@@ -11847,7 +11847,7 @@
       </c>
       <c r="J24" s="25">
         <f>(J22/(J13*9.8))*100</f>
-        <v>76.978021978021971</v>
+        <v>75.164835164835168</v>
       </c>
       <c r="K24" s="24" t="s">
         <v>234</v>
@@ -11869,7 +11869,7 @@
       </c>
       <c r="J25" s="25">
         <f>(J23/(J13*9.8))*100</f>
-        <v>23.021978021978022</v>
+        <v>24.835164835164836</v>
       </c>
       <c r="K25" s="24" t="s">
         <v>234</v>
@@ -11908,7 +11908,7 @@
       </c>
       <c r="J27" s="25">
         <f>J22*(J18/2000)*J17</f>
-        <v>1054.4948432276758</v>
+        <v>965.30309524589188</v>
       </c>
       <c r="K27" s="24" t="s">
         <v>240</v>
@@ -11930,7 +11930,7 @@
       </c>
       <c r="J28" s="25">
         <f>J23*(J18/2000)*J17</f>
-        <v>315.36997809592879</v>
+        <v>318.94517474498764</v>
       </c>
       <c r="K28" s="24" t="s">
         <v>240</v>
@@ -12228,7 +12228,7 @@
       </c>
       <c r="J44" s="25">
         <f>2*J33*(J50*6894.76)*(J36*0.0254^2)*(J35/1000)</f>
-        <v>527.24742161383801</v>
+        <v>482.651547622946</v>
       </c>
       <c r="K44" s="24" t="s">
         <v>240</v>
@@ -12250,7 +12250,7 @@
       </c>
       <c r="J45" s="25">
         <f>2*J34*(J51*6894.76)*(J37*0.0254^2)*(J35/1000)</f>
-        <v>157.68498904796439</v>
+        <v>159.47258737249385</v>
       </c>
       <c r="K45" s="24" t="s">
         <v>240</v>
@@ -12357,7 +12357,7 @@
       </c>
       <c r="J50" s="25">
         <f>(J27/2)/(2*J33*(J35/1000)*J46)/6894.76</f>
-        <v>1115.3444846345299</v>
+        <v>1021.0059254416738</v>
       </c>
       <c r="K50" s="24" t="s">
         <v>325</v>
@@ -12369,7 +12369,7 @@
       </c>
       <c r="J51" s="25">
         <f>(J28/2)/(2*J34*(J35/1000)*J47)/6894.76</f>
-        <v>333.56840761018418</v>
+        <v>337.34991103774598</v>
       </c>
       <c r="K51" s="24" t="s">
         <v>325</v>
@@ -12427,7 +12427,7 @@
       </c>
       <c r="J54" s="25">
         <f>J50*6894.76*J48/(J40*J41)</f>
-        <v>1217.6865631103099</v>
+        <v>1114.691661091344</v>
       </c>
       <c r="K54" s="24" t="s">
         <v>227</v>
@@ -12449,7 +12449,7 @@
       </c>
       <c r="J55" s="25">
         <f>J51*6894.76*J49/(J40*(1-J41))</f>
-        <v>546.26410058160582</v>
+        <v>552.45683203211331</v>
       </c>
       <c r="K55" s="24" t="s">
         <v>227</v>
@@ -12471,7 +12471,7 @@
       </c>
       <c r="J56" s="25">
         <f>MAX(J54,J55)</f>
-        <v>1217.6865631103099</v>
+        <v>1114.691661091344</v>
       </c>
       <c r="K56" s="24" t="s">
         <v>227</v>

</xml_diff>